<commit_message>
docs: smoke de los 5 paises + hallazgos de ruido y costo de compute
Los 5 paises corrieron sin errores (england 5min, france 6.4h, germany 3.3h,
italy 8.4h, spain 7.1h; 25.3h de compute total). Resultados y los 2 hallazgos
que condicionan el plan de mejoras, en docs/REFACTOR.md:

1. La metrica tiene mas ruido que las mejoras a testear: 6 corridas con config
   identica dieron f1 entre 40.0 y 45.0 y ROI entre -50.6 y -19.2, porque
   RandomUnderSampler/RandomOverSampler se instancian sin random_state. La
   tabla por pais NO es un ranking.
2. El costo se paga una vez por (pais, iteration_date), no por corrida: 3-8h
   la primera vez (mapeo global de sofifa ~1h28 + formateo ~1h48, ambos
   parseo de .xlsx) contra 5 min con la cache del dia ya armada. Aplicar
   Parquet a los crudos es la palanca de performance mas grande que queda.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/_shared/logs/_training_log.xlsx
+++ b/data/_shared/logs/_training_log.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1120,6 +1120,346 @@
         <v>-77.54048531187325</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:15:23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>16617e5fe</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>./data/england/modeling/2026-09-11/models</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>41.37254901960785</v>
+      </c>
+      <c r="L11" t="n">
+        <v>41.37254901960785</v>
+      </c>
+      <c r="M11" t="n">
+        <v>46.46464646464646</v>
+      </c>
+      <c r="N11" t="n">
+        <v>46.46464646464646</v>
+      </c>
+      <c r="O11" t="n">
+        <v>-47.14836589374595</v>
+      </c>
+      <c r="P11" t="n">
+        <v>-47.14836589374595</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>-53.67111036603984</v>
+      </c>
+      <c r="R11" t="n">
+        <v>-53.67111036603984</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-12T01:38:17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>16617e5fe</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>382.9</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>./data/france/modeling/2026-09-11/models</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>37.14497687003578</v>
+      </c>
+      <c r="L12" t="n">
+        <v>37.14497687003578</v>
+      </c>
+      <c r="M12" t="n">
+        <v>45.16129032258064</v>
+      </c>
+      <c r="N12" t="n">
+        <v>45.16129032258064</v>
+      </c>
+      <c r="O12" t="n">
+        <v>-60.50308245296514</v>
+      </c>
+      <c r="P12" t="n">
+        <v>-60.50308245296514</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>-34.97755389353787</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-34.97755389353787</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-12T22:58:54</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ac26402b6</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>germany</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>197.2</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>./data/germany/modeling/2026-09-12/models</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>43.75503626107977</v>
+      </c>
+      <c r="L13" t="n">
+        <v>43.75503626107977</v>
+      </c>
+      <c r="M13" t="n">
+        <v>50</v>
+      </c>
+      <c r="N13" t="n">
+        <v>50</v>
+      </c>
+      <c r="O13" t="n">
+        <v>-8.650800081887255</v>
+      </c>
+      <c r="P13" t="n">
+        <v>-8.650800081887255</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>15.82003802326102</v>
+      </c>
+      <c r="R13" t="n">
+        <v>15.82003802326102</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-13T07:22:24</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ac26402b6</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>503.4</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>./data/italy/modeling/2026-09-12/models</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>48.03436743489637</v>
+      </c>
+      <c r="L14" t="n">
+        <v>48.03436743489637</v>
+      </c>
+      <c r="M14" t="n">
+        <v>54</v>
+      </c>
+      <c r="N14" t="n">
+        <v>54</v>
+      </c>
+      <c r="O14" t="n">
+        <v>7.559487539008643</v>
+      </c>
+      <c r="P14" t="n">
+        <v>7.559487539008643</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>-9.541295311183561</v>
+      </c>
+      <c r="R14" t="n">
+        <v>-9.541295311183561</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-13T14:29:36</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ac26402b6</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>spain</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>427.2</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>./data/spain/modeling/2026-09-13/models</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>43.82645803698435</v>
+      </c>
+      <c r="L15" t="n">
+        <v>43.82645803698435</v>
+      </c>
+      <c r="M15" t="n">
+        <v>51</v>
+      </c>
+      <c r="N15" t="n">
+        <v>51</v>
+      </c>
+      <c r="O15" t="n">
+        <v>-15.30496264986677</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-15.30496264986677</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>-35.03462237398661</v>
+      </c>
+      <c r="R15" t="n">
+        <v>-35.03462237398661</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>